<commit_message>
feat(cmdb-import): read the CMDB sheets, key on APPID, owner from Applicatie Eigenaar (Persoon)
After the review with Gemeente Rotterdam the import reads the derived
sheets "Onbeh Applicaties CMDB" (applications without arranged
maintenance) and "Beheerde Applicaties CMDB" (with maintenance)
instead of the raw TOPdesk input sheets. Modules are matched on
topdesk:<municipality>:<APPID>; Applicatie Code becomes externalId.
Formula cells contribute their cached value; a missing cached value
gives an empty field and a row warning. The owner comes from
"Applicatie Eigenaar (Persoon)" with its function as role; the
technical-owner pack is removed. Applicatiesoort, BNN Classificatie,
Classificatie (TIME) and End-of-Life Functioneel are mapped with
configurable placeholder values. A test asserts that person data is
never anonymously readable.

Jira: https://conduction.atlassian.net/browse/WOO-586

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/cmdb/topdesk-export-anonymised.xlsx
+++ b/tests/fixtures/cmdb/topdesk-export-anonymised.xlsx
@@ -33928,7 +33928,7 @@
       </c>
       <c r="E2" s="17" t="str">
         <f>'Invoer AIA data'!W2</f>
-        <v/>
+        <v>Mailen</v>
       </c>
       <c r="F2" s="17" t="str">
         <f>'Invoer AIA data'!AU2</f>
@@ -34005,7 +34005,7 @@
       </c>
       <c r="AE2" s="17" t="str">
         <f>'Invoer AIA data'!AN2</f>
-        <v/>
+        <v>Herbeoordeling</v>
       </c>
       <c r="AF2" s="18">
         <f>'Invoer AIA data'!E2</f>
@@ -34017,11 +34017,11 @@
       </c>
       <c r="AH2" s="17" t="str">
         <f>'Invoer AIA data'!AJ2</f>
-        <v/>
+        <v>Ja</v>
       </c>
       <c r="AI2" s="17" t="str">
         <f>'Invoer AIA data'!AO2</f>
-        <v/>
+        <v>Geen</v>
       </c>
     </row>
     <row r="3" spans="1:35" x14ac:dyDescent="0.25">
@@ -47622,7 +47622,7 @@
       </c>
       <c r="E2" s="28" t="str">
         <f>'Invoer APP data'!AA2</f>
-        <v/>
+        <v>Naamtest</v>
       </c>
       <c r="F2" s="17" t="str">
         <f>IF('Invoer APP data'!BH2="Ja","Ja","Nee")</f>
@@ -47638,7 +47638,7 @@
       </c>
       <c r="I2" s="28" t="str">
         <f>'Invoer APP data'!AD2</f>
-        <v/>
+        <v>Saas</v>
       </c>
       <c r="J2" s="18">
         <f>IF('Invoer APP data'!S2=73050,49675,'Invoer APP data'!S2)</f>
@@ -47650,11 +47650,11 @@
       </c>
       <c r="L2" s="17" t="str">
         <f>'Invoer APP data'!K2</f>
-        <v/>
+        <v>Teamleider Applicatiebeheer</v>
       </c>
       <c r="M2" s="17" t="str">
         <f>IF('Invoer APP data'!Q2="",'Invoer APP data'!K2,'Invoer APP data'!Q2)</f>
-        <v/>
+        <v>Teamleider Applicatiebeheer</v>
       </c>
       <c r="N2" s="17" t="str">
         <f>IF('Invoer APP data'!AH2 = "","Niet bekend",MID('Invoer APP data'!AH2,5,25))</f>
@@ -47713,7 +47713,7 @@
       </c>
       <c r="AB2" s="17" t="str">
         <f>IF('Invoer APP data'!AD2="Saas","Ja","Nee")</f>
-        <v>Nee</v>
+        <v>Ja</v>
       </c>
       <c r="AC2" s="17" t="str">
         <f>'Invoer APP data'!AU2</f>
@@ -47729,7 +47729,7 @@
       </c>
       <c r="AF2" s="17" t="str">
         <f>'Invoer APP data'!BD2</f>
-        <v/>
+        <v>Herbeoordeling</v>
       </c>
       <c r="AG2" s="18">
         <f>'Invoer APP data'!E2</f>
@@ -47737,15 +47737,20 @@
       </c>
       <c r="AH2" s="18" t="str">
         <f>IF('Invoer APP data'!AK2="","NB",'Invoer APP data'!AK2)</f>
-        <v>NB</v>
+        <v>BBN2</v>
       </c>
       <c r="AI2" s="18" t="str">
         <f>'Invoer APP data'!AX2</f>
-        <v/>
+        <v>Ja</v>
       </c>
       <c r="AJ2" s="17" t="str">
         <f>'Invoer APP data'!M2</f>
         <v>ICT AB CD Test123</v>
+      </c>
+      <c r="AM2" t="inlineStr">
+        <is>
+          <t>NT123</t>
+        </is>
       </c>
     </row>
     <row r="3" spans="1:42" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
fix(cmdb-import): strip printer settings, dates and revision ids from the fixtures
Four of the five CMDB fixtures still carried the printer settings of every
sheet (naming the printers of the machine the export was handled on), the
creation date of the original export, the workbook's revision GUID and the
filter ranges and sort orders that record the size of the original data.

build-fixtures.py now always sanitises the committed export (idempotent):
it drops xl/printerSettings/ with its relationships, pageSetup links and
content type, empties the document properties in core.xml and app.xml,
sets both dates to a fixed neutral date, removes the revision pointer and
the xr uid attributes, the _FilterDatabase names and sort states, and
narrows auto filters to the header row. The five fixtures are regenerated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/cmdb/topdesk-export-anonymised.xlsx
+++ b/tests/fixtures/cmdb/topdesk-export-anonymised.xlsx
@@ -3,9 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CAEA186-9AA1-40C3-AE4A-D564E2BAA450}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="51480" yWindow="5280" windowWidth="29040" windowHeight="15840" tabRatio="594" firstSheet="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="51480" yWindow="5280" windowWidth="29040" windowHeight="15840" tabRatio="594" firstSheet="1"/>
   </bookViews>
   <sheets>
     <sheet name="Invoer AIA data" sheetId="6" r:id="rId1"/>
@@ -19,18 +18,6 @@
     <sheet name="Blad3" sheetId="4" r:id="rId9"/>
     <sheet name="Origineel" sheetId="1" r:id="rId10"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">Behandelgroepen!$A$1:$E$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Beheerde Applicaties CMDB'!$A$1:$AP$1066</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">Blad3!$A$1:$A$128</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Gearchiveerde Applicaties'!$A$1:$I$434</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Invoer AIA data'!$A$1:$BB$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Invoer APP data'!$A$1:$CD$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Invoer gearchiveerde appl'!$A$1:$CO$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Onbeh Applicaties CMDB'!$A$1:$AH$98</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">Origineel!$A$2:$AA$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Relatie APP oplosgroepen'!$B$2:$APJ$2</definedName>
-  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -1363,7 +1350,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C8FFAE6-2986-4F38-9797-2552E7727FDA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:AZ249"/>
   <sheetFormatPr defaultColWidth="20.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2708,17 +2695,17 @@
       <c r="C249" s="13"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BB1" xr:uid="{6C8FFAE6-2986-4F38-9797-2552E7727FDA}"/>
+  <autoFilter ref="A1:BB1"/>
   <hyperlinks>
-    <hyperlink ref="J2" r:id="rId1" display="mailto:letter.achternaam@gemeente.nl" xr:uid="{92E263F2-1000-4547-B807-F14BED24D8E1}"/>
+    <hyperlink ref="J2" r:id="rId1" display="mailto:letter.achternaam@gemeente.nl"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:AA1141"/>
   <sheetFormatPr defaultColWidth="214.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -33755,14 +33742,14 @@
       <c r="AA1141" s="10"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:AA2" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A2:AA2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2F26ADF-A76E-483E-B515-1BC07834D443}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:AI100"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -34417,9 +34404,9 @@
       <c r="AF100" s="18"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AH98" xr:uid="{B2F26ADF-A76E-483E-B515-1BC07834D443}"/>
+  <autoFilter ref="A1:AH1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
   <ignoredErrors>
     <ignoredError xmlns:x16r3="http://schemas.microsoft.com/office/spreadsheetml/2018/08/main" sqref="AF2" x16r3:misleadingFormat="1"/>
   </ignoredErrors>
@@ -34427,7 +34414,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C7279925-5FC1-4109-A23D-8ADA8308449E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:CD1136"/>
   <sheetFormatPr defaultColWidth="27.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -47418,18 +47405,18 @@
       <c r="AD1136" s="11"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:CD1" xr:uid="{C7279925-5FC1-4109-A23D-8ADA8308449E}"/>
+  <autoFilter ref="A1:CD1"/>
   <hyperlinks>
-    <hyperlink ref="O2" r:id="rId1" xr:uid="{7EFA633E-E1C5-4984-B2ED-623F21986EA4}"/>
-    <hyperlink ref="U2" r:id="rId2" xr:uid="{56D610AE-976A-4756-8D98-54457789B785}"/>
+    <hyperlink ref="O2" r:id="rId1"/>
+    <hyperlink ref="U2" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5FA9F2C5-2A80-40F0-ABC6-EC876C3BEE48}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:AP1068"/>
   <sheetFormatPr defaultColWidth="45.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -57367,19 +57354,15 @@
       <c r="Y1068" s="18"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AP1066" xr:uid="{5FA9F2C5-2A80-40F0-ABC6-EC876C3BEE48}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A852:AP852">
-      <sortCondition ref="K1:K1062"/>
-    </sortState>
-  </autoFilter>
+  <autoFilter ref="A1:AP1"/>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA4764C0-EEB6-43A1-977A-04CBD0DD848C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:CO2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -58040,21 +58023,21 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:CO1" xr:uid="{CA4764C0-EEB6-43A1-977A-04CBD0DD848C}"/>
+  <autoFilter ref="A1:CO1"/>
   <phoneticPr fontId="3" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="J2" r:id="rId1" display="mailto:letter.achternaam@gemeente.nl" xr:uid="{1B6002AF-D815-4999-B25E-78F8BBCD6D43}"/>
-    <hyperlink ref="O2" r:id="rId2" display="mailto:letter.achternaam@gemeente.nl" xr:uid="{95346917-3E80-4EA3-A1B1-C4C7E6722FC6}"/>
-    <hyperlink ref="P2" r:id="rId3" xr:uid="{66E98122-A82B-4238-940E-1F641D831B4C}"/>
-    <hyperlink ref="U2" r:id="rId4" display="mailto:letter.achternaam@gemeente.nl" xr:uid="{46576A51-1928-42FD-8F76-9ACFEE814F94}"/>
+    <hyperlink ref="J2" r:id="rId1" display="mailto:letter.achternaam@gemeente.nl"/>
+    <hyperlink ref="O2" r:id="rId2" display="mailto:letter.achternaam@gemeente.nl"/>
+    <hyperlink ref="P2" r:id="rId3"/>
+    <hyperlink ref="U2" r:id="rId4" display="mailto:letter.achternaam@gemeente.nl"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="360" verticalDpi="360"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F31C3127-42FF-46D7-A7BE-D6B327F344FD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:I466"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -59992,14 +59975,14 @@
       <c r="I466" s="27"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I434" xr:uid="{F31C3127-42FF-46D7-A7BE-D6B327F344FD}"/>
+  <autoFilter ref="A1:I1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="360" verticalDpi="360"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4C58AFA-DED0-476A-AD3C-1E5843262B11}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:AMY3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -63147,14 +63130,14 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B2:APJ2" xr:uid="{D4C58AFA-DED0-476A-AD3C-1E5843262B11}"/>
+  <autoFilter ref="B2:APJ2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE148F3A-2307-4656-B058-576ECC862847}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:D1095"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -66603,18 +66586,14 @@
       <c r="A1095"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E98" xr:uid="{FE148F3A-2307-4656-B058-576ECC862847}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D98">
-      <sortCondition ref="A1:A98"/>
-    </sortState>
-  </autoFilter>
+  <autoFilter ref="A1:E1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5015BD4B-87F1-492F-B21B-0961C7B7BBA9}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:P2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -66654,12 +66633,8 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:A128" xr:uid="{5015BD4B-87F1-492F-B21B-0961C7B7BBA9}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:A128">
-      <sortCondition ref="A1:A128"/>
-    </sortState>
-  </autoFilter>
+  <autoFilter ref="A1:A1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
</xml_diff>